<commit_message>
Fix payment date to anchor off adjusted period end (Bloomberg standard)
Payment date T+N was incorrectly counted from the unadjusted period end,
deviating from Bloomberg SWPM / ISDA convention by 1 day whenever a period
end falls on a weekend or holiday.

Example: unadjusted end Sunday May 10, ModifiedFollowing -> Monday May 11.
  Old (bug): T+2 from Sunday May 10 -> Tuesday May 12
  New (fix): T+2 from Monday May 11 -> Wednesday May 13

Changes:
- schedule.py line 225: u_e -> a_e as the payment anchor
- test_schedule.py: new test covering a monthly period ending on Sunday Nov 1
  2026, asserting payment = Wed Nov 4 (not Tue Nov 3)
- schema.md: update payment delay description
- Convention_Reference.xlsx / build script: update delay field description

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Convention_Reference.xlsx
+++ b/Convention_Reference.xlsx
@@ -1151,7 +1151,8 @@
       <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Business days after the accrual period ends before the coupon is paid.
-0 = pay on the last day of the period</t>
+T+N is counted from the ADJUSTED period end (Bloomberg/ISDA standard).
+0 = pay on the last day of the adjusted period</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1567,8 @@
       <c r="F34" s="5" t="inlineStr">
         <is>
           <t>Business days after the compounding period ends before the floating coupon is settled.
-Payment date = unadjusted period end + delay, then rolled by floating_pay_date_adj</t>
+T+N is counted from the ADJUSTED period end (Bloomberg/ISDA standard), then rolled by floating_pay_date_adj.
+Example: period ends Sunday May 10 -&gt; adjusts to Monday May 11 -&gt; T+2 = Wednesday May 13</t>
         </is>
       </c>
     </row>

</xml_diff>